<commit_message>
alignment and fixed testc ases
</commit_message>
<xml_diff>
--- a/src/main/resources/SubrecipientContact_Field_Values.xlsx
+++ b/src/main/resources/SubrecipientContact_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21601"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22527"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86205E03-71D1-44CD-AC25-3FDAD4692CB5}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A90ED4CD-E9A2-407C-B7C0-D3C09F692D58}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{9C2C5CEA-7821-409A-A434-0BC7CE36CBA3}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{9C2C5CEA-7821-409A-A434-0BC7CE36CBA3}"/>
   </bookViews>
   <sheets>
     <sheet name="Creation" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Refactored Announcement module, Completed 7 scenarios for user registration
</commit_message>
<xml_diff>
--- a/src/main/resources/SubrecipientContact_Field_Values.xlsx
+++ b/src/main/resources/SubrecipientContact_Field_Values.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22624"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23029"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MCPL#L92\Desktop\Automation projects\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workpace-gov-grants-framework-automation\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1BAE9D6-5462-4D85-8B9F-6D5663517BD2}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3695D3BA-E324-449C-89ED-F4A9E0BB13F6}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="11949" xr2:uid="{9C2C5CEA-7821-409A-A434-0BC7CE36CBA3}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10395" xr2:uid="{9C2C5CEA-7821-409A-A434-0BC7CE36CBA3}"/>
   </bookViews>
   <sheets>
     <sheet name="Creation" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="26">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -60,9 +60,6 @@
     <t>Phone</t>
   </si>
   <si>
-    <t>AccountId</t>
-  </si>
-  <si>
     <t>Primary</t>
   </si>
   <si>
@@ -75,9 +72,6 @@
     <t>Legal Contact</t>
   </si>
   <si>
-    <t>Automation.manager@yopmail.com</t>
-  </si>
-  <si>
     <t>704-777-(7868)</t>
   </si>
   <si>
@@ -105,9 +99,6 @@
     <t>USA</t>
   </si>
   <si>
-    <t>SAN DIEGO ELECTRICAL TRAINING TRUST</t>
-  </si>
-  <si>
     <t>ContactTypeInternal__c</t>
   </si>
   <si>
@@ -115,6 +106,9 @@
   </si>
   <si>
     <t>Automation Runtime Contact</t>
+  </si>
+  <si>
+    <t>AutomationManager@yopmail.com</t>
   </si>
 </sst>
 </file>
@@ -487,16 +481,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17D21291-1546-4312-AD3E-AC2481560893}">
-  <dimension ref="A1:C12"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <dimension ref="A1:C11"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="17.4609375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.3046875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="35.4609375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.07421875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.46484375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.46484375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.06640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -507,7 +501,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -515,10 +509,10 @@
         <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -526,10 +520,10 @@
         <v>5</v>
       </c>
       <c r="C3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -537,95 +531,84 @@
         <v>4</v>
       </c>
       <c r="C4" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" t="s">
-        <v>8</v>
-      </c>
-      <c r="C6" s="2" t="s">
+      <c r="C7" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A7" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" t="s">
-        <v>7</v>
-      </c>
-      <c r="C7" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A8" t="s">
-        <v>3</v>
-      </c>
-      <c r="B8" t="s">
+      <c r="C8" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" t="s">
         <v>16</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C9" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C10">
+        <v>20171</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A11" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11" t="s">
         <v>21</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B9" t="s">
-        <v>17</v>
-      </c>
-      <c r="C9" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A10" t="s">
-        <v>3</v>
-      </c>
-      <c r="B10" t="s">
-        <v>18</v>
-      </c>
-      <c r="C10" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A11" t="s">
-        <v>3</v>
-      </c>
-      <c r="B11" t="s">
-        <v>19</v>
-      </c>
-      <c r="C11">
-        <v>20171</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A12" t="s">
-        <v>3</v>
-      </c>
-      <c r="B12" t="s">
-        <v>20</v>
-      </c>
-      <c r="C12" t="s">
-        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -640,13 +623,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{321AD5C1-CFBB-4EF4-9C99-C433DBDD2201}">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="14.3046875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.765625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.73046875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -657,26 +640,26 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>3</v>
       </c>
       <c r="B2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" t="s">
         <v>11</v>
       </c>
-      <c r="C2" t="s">
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3" t="s">
         <v>12</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="C3" t="s">
-        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
1.Completed 12 scenarios for closeout module 2. Modification as per failure in regression run.
</commit_message>
<xml_diff>
--- a/src/main/resources/SubrecipientContact_Field_Values.xlsx
+++ b/src/main/resources/SubrecipientContact_Field_Values.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workpace-gov-grants-framework-automation\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3695D3BA-E324-449C-89ED-F4A9E0BB13F6}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24E82C6B-DADB-47CF-A938-35001D10BFF2}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="10395" xr2:uid="{9C2C5CEA-7821-409A-A434-0BC7CE36CBA3}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="28">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -109,13 +109,19 @@
   </si>
   <si>
     <t>AutomationManager@yopmail.com</t>
+  </si>
+  <si>
+    <t>fieldAccountId</t>
+  </si>
+  <si>
+    <t>SAN DIEGO ELECTRICAL TRAINING TRUST</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -133,6 +139,12 @@
     </font>
     <font>
       <sz val="7"/>
+      <color rgb="FF222222"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="5"/>
       <color rgb="FF222222"/>
       <name val="Consolas"/>
       <family val="3"/>
@@ -159,13 +171,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -481,7 +494,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17D21291-1546-4312-AD3E-AC2481560893}">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="17.46484375" bestFit="1" customWidth="1"/>
@@ -506,10 +519,10 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" t="s">
-        <v>24</v>
+        <v>26</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.45">
@@ -517,10 +530,10 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.45">
@@ -528,10 +541,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>25</v>
+        <v>5</v>
+      </c>
+      <c r="C4" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.45">
@@ -539,10 +552,10 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>13</v>
+        <v>4</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.45">
@@ -550,10 +563,10 @@
         <v>3</v>
       </c>
       <c r="B6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C6" t="s">
-        <v>9</v>
+        <v>8</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.45">
@@ -561,10 +574,10 @@
         <v>3</v>
       </c>
       <c r="B7" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="C7" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.45">
@@ -572,7 +585,7 @@
         <v>3</v>
       </c>
       <c r="B8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C8" t="s">
         <v>19</v>
@@ -583,10 +596,10 @@
         <v>3</v>
       </c>
       <c r="B9" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.45">
@@ -594,10 +607,10 @@
         <v>3</v>
       </c>
       <c r="B10" t="s">
-        <v>17</v>
-      </c>
-      <c r="C10">
-        <v>20171</v>
+        <v>16</v>
+      </c>
+      <c r="C10" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.45">
@@ -605,15 +618,26 @@
         <v>3</v>
       </c>
       <c r="B11" t="s">
+        <v>17</v>
+      </c>
+      <c r="C11">
+        <v>20171</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A12" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" t="s">
         <v>18</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C12" t="s">
         <v>21</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C4" r:id="rId1" xr:uid="{908A1EC6-29F1-48F2-9098-0E2D16D0C72E}"/>
+    <hyperlink ref="C5" r:id="rId1" xr:uid="{908A1EC6-29F1-48F2-9098-0E2D16D0C72E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="200" verticalDpi="200" r:id="rId2"/>

</xml_diff>